<commit_message>
Condition and logic functions
</commit_message>
<xml_diff>
--- a/04_ConditionAndLogic.xlsx
+++ b/04_ConditionAndLogic.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f595840ab58673e5/Desktop/Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{04659108-64AA-4C60-8BCB-49B366B2B693}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{343A5D57-E0CD-4CD9-9FC2-D714DD9CE36D}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{04659108-64AA-4C60-8BCB-49B366B2B693}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{38C5DDB7-1963-4958-853E-CC1FF5032288}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="4080" yWindow="4080" windowWidth="17280" windowHeight="9960" xr2:uid="{DB4AE30E-C932-48ED-8470-9F4863C0E4DD}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{DB4AE30E-C932-48ED-8470-9F4863C0E4DD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="27">
   <si>
     <t>Full Name</t>
   </si>
@@ -94,9 +94,6 @@
   </si>
   <si>
     <t>eva@example.com</t>
-  </si>
-  <si>
-    <t>Salary Status</t>
   </si>
   <si>
     <t>Rating</t>
@@ -549,9 +546,7 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="4" t="s">
-        <v>22</v>
-      </c>
+      <c r="J1" s="4"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
@@ -703,16 +698,16 @@
         <v>5</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C10" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="E10" s="4" t="s">
         <v>24</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
@@ -820,7 +815,7 @@
         <v>2</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">

</xml_diff>